<commit_message>
Version 1.2 de SGA Laboratorio
</commit_message>
<xml_diff>
--- a/modules/laboratorio/muestra/plantilla/CSJ-DRDYCS-LAYS – R - 1-RESULTADOS ANALISIS DE  SUELOS.xlsx
+++ b/modules/laboratorio/muestra/plantilla/CSJ-DRDYCS-LAYS – R - 1-RESULTADOS ANALISIS DE  SUELOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SISTEMAS\gestionTI2026\modules\laboratorio\muestra\plantilla\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB00C35-1BF6-49CF-803B-1A98CE239B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678C2917-050B-4645-B4D5-5DAE53521E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -197,19 +197,19 @@
     <t>CSJ-DRDYCS-LAYS – R - 1</t>
   </si>
   <si>
-    <t>Ms.C. Ing. Fiorella Gamarra Quipas</t>
-  </si>
-  <si>
     <t>RESPONSABLE LABORATORIO AGUAS Y SUELOS PECH</t>
   </si>
   <si>
-    <t xml:space="preserve">Ms.C.Mblgo.Rosa Anais Baca Ardiles </t>
-  </si>
-  <si>
     <t>CBP: 10659</t>
   </si>
   <si>
     <t>OTROS</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
 </sst>
 </file>
@@ -812,13 +812,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1473,105 +1470,105 @@
   <dimension ref="A2:X66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" style="7" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" style="7" customWidth="1"/>
-    <col min="5" max="5" width="9.28515625" style="7" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" style="7" customWidth="1"/>
-    <col min="7" max="9" width="10.85546875" style="7" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" style="7" customWidth="1"/>
-    <col min="12" max="12" width="6.28515625" style="7" customWidth="1"/>
-    <col min="13" max="16384" width="11.42578125" style="7"/>
+    <col min="1" max="1" width="4.5703125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" style="6" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" style="6" customWidth="1"/>
+    <col min="7" max="9" width="10.85546875" style="6" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" style="6" customWidth="1"/>
+    <col min="12" max="12" width="6.28515625" style="6" customWidth="1"/>
+    <col min="13" max="16384" width="11.42578125" style="6"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="6" t="s">
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="66" t="s">
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="67"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="3" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="6" t="s">
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="68"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="67"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
     </row>
     <row r="6" spans="1:12" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:12" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="B7" s="69" t="s">
+      <c r="B7" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="69"/>
-      <c r="D7" s="69"/>
-      <c r="E7" s="69"/>
-      <c r="F7" s="69"/>
-      <c r="G7" s="69"/>
-      <c r="H7" s="69"/>
-      <c r="I7" s="69"/>
-      <c r="J7" s="69"/>
-      <c r="K7" s="69"/>
+      <c r="C7" s="68"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="68"/>
+      <c r="H7" s="68"/>
+      <c r="I7" s="68"/>
+      <c r="J7" s="68"/>
+      <c r="K7" s="68"/>
     </row>
     <row r="8" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="62" t="s">
+      <c r="A8" s="9"/>
+      <c r="B8" s="61" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="62"/>
-      <c r="H8" s="62"/>
-      <c r="I8" s="62"/>
-      <c r="J8" s="62"/>
-      <c r="K8" s="62"/>
-      <c r="L8" s="10"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+      <c r="I8" s="61"/>
+      <c r="J8" s="61"/>
+      <c r="K8" s="61"/>
+      <c r="L8" s="9"/>
     </row>
     <row r="9" spans="1:12" ht="7.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -1579,812 +1576,812 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
-      <c r="L9" s="10"/>
+      <c r="L9" s="9"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="56" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="57"/>
+      <c r="C10" s="56"/>
       <c r="D10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E10" s="3"/>
+      <c r="E10" s="2"/>
       <c r="F10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" s="2"/>
       <c r="H10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I10" s="3"/>
+      <c r="I10" s="2"/>
       <c r="J10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K10" s="3"/>
-      <c r="L10" s="10"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="9"/>
     </row>
     <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
       <c r="D11" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
+        <v>46</v>
+      </c>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
     </row>
     <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="10"/>
-      <c r="B12" s="56" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="58"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="61"/>
-      <c r="L12" s="10"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="58"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="60"/>
+      <c r="L12" s="9"/>
     </row>
     <row r="13" spans="1:12" ht="4.1500000000000004" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
     </row>
     <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="56" t="s">
+      <c r="A14" s="9"/>
+      <c r="B14" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="58"/>
-      <c r="D14" s="62" t="s">
+      <c r="C14" s="57"/>
+      <c r="D14" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="62"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="62" t="s">
+      <c r="E14" s="61"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="61" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="62"/>
-      <c r="I14" s="3"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="2"/>
       <c r="J14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K14" s="3"/>
-      <c r="L14" s="10"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="9"/>
     </row>
     <row r="15" spans="1:12" ht="4.1500000000000004" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
     </row>
     <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="56" t="s">
+      <c r="A16" s="9"/>
+      <c r="B16" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="58"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
-      <c r="H16" s="60"/>
-      <c r="I16" s="60"/>
-      <c r="J16" s="60"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="10"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="59"/>
+      <c r="G16" s="59"/>
+      <c r="H16" s="59"/>
+      <c r="I16" s="59"/>
+      <c r="J16" s="59"/>
+      <c r="K16" s="60"/>
+      <c r="L16" s="9"/>
     </row>
     <row r="17" spans="1:12" ht="3" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
     </row>
     <row r="18" spans="1:12" ht="13.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
-      <c r="B18" s="56" t="s">
+      <c r="A18" s="9"/>
+      <c r="B18" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="19" t="s">
+      <c r="C18" s="56"/>
+      <c r="D18" s="18" t="s">
         <v>32</v>
       </c>
       <c r="E18" s="2"/>
-      <c r="F18" s="64" t="s">
+      <c r="F18" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="G18" s="65"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="64" t="s">
+      <c r="G18" s="64"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="J18" s="65"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="10"/>
+      <c r="J18" s="64"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="9"/>
     </row>
     <row r="19" spans="1:12" ht="3" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
     </row>
     <row r="20" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
-      <c r="B20" s="56" t="s">
+      <c r="A20" s="9"/>
+      <c r="B20" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="58"/>
-      <c r="D20" s="59"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="63" t="s">
+      <c r="C20" s="57"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="63"/>
-      <c r="H20" s="63"/>
-      <c r="I20" s="63"/>
-      <c r="J20" s="60"/>
-      <c r="K20" s="60"/>
-      <c r="L20" s="10"/>
+      <c r="G20" s="62"/>
+      <c r="H20" s="62"/>
+      <c r="I20" s="62"/>
+      <c r="J20" s="59"/>
+      <c r="K20" s="59"/>
+      <c r="L20" s="9"/>
     </row>
     <row r="21" spans="1:12" ht="4.1500000000000004" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10"/>
-      <c r="B22" s="56" t="s">
+      <c r="A22" s="9"/>
+      <c r="B22" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="57"/>
-      <c r="D22" s="15" t="s">
+      <c r="C22" s="56"/>
+      <c r="D22" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="59"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="16" t="s">
+      <c r="E22" s="58"/>
+      <c r="F22" s="59"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="10"/>
+      <c r="I22" s="59"/>
+      <c r="J22" s="59"/>
+      <c r="K22" s="59"/>
+      <c r="L22" s="9"/>
     </row>
     <row r="23" spans="1:12" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
     </row>
     <row r="24" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10"/>
-      <c r="B24" s="70" t="s">
+      <c r="A24" s="9"/>
+      <c r="B24" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="71"/>
-      <c r="D24" s="81" t="s">
+      <c r="C24" s="70"/>
+      <c r="D24" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="81"/>
-      <c r="F24" s="81"/>
-      <c r="G24" s="48" t="s">
+      <c r="E24" s="80"/>
+      <c r="F24" s="80"/>
+      <c r="G24" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="H24" s="50" t="s">
+      <c r="H24" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="51"/>
-      <c r="J24" s="50" t="s">
+      <c r="I24" s="50"/>
+      <c r="J24" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="K24" s="74"/>
-      <c r="L24" s="10"/>
+      <c r="K24" s="73"/>
+      <c r="L24" s="9"/>
     </row>
     <row r="25" spans="1:12" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="72"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
-      <c r="F25" s="82"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="52"/>
-      <c r="I25" s="53"/>
-      <c r="J25" s="52"/>
-      <c r="K25" s="75"/>
-      <c r="L25" s="10"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="71"/>
+      <c r="C25" s="72"/>
+      <c r="D25" s="81"/>
+      <c r="E25" s="81"/>
+      <c r="F25" s="81"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="51"/>
+      <c r="I25" s="52"/>
+      <c r="J25" s="51"/>
+      <c r="K25" s="74"/>
+      <c r="L25" s="9"/>
     </row>
     <row r="26" spans="1:12" ht="2.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="10"/>
-      <c r="B27" s="43" t="s">
+      <c r="A27" s="9"/>
+      <c r="B27" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="44"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="83"/>
-      <c r="F27" s="83"/>
-      <c r="G27" s="83"/>
-      <c r="H27" s="83"/>
-      <c r="I27" s="83"/>
-      <c r="J27" s="83"/>
-      <c r="K27" s="83"/>
-      <c r="L27" s="10"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="82"/>
+      <c r="J27" s="82"/>
+      <c r="K27" s="82"/>
+      <c r="L27" s="9"/>
     </row>
     <row r="28" spans="1:12" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10"/>
-      <c r="L28" s="10"/>
-    </row>
-    <row r="29" spans="1:12" s="5" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11"/>
-      <c r="B29" s="38"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="54"/>
-      <c r="I29" s="55"/>
-      <c r="J29" s="25"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="10"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" s="4" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="45"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="53"/>
+      <c r="I29" s="54"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="9"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="10"/>
-      <c r="B30" s="38"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="39"/>
-      <c r="I30" s="40"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="10"/>
+      <c r="A30" s="9"/>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="45"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="39"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="9"/>
     </row>
     <row r="31" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
-      <c r="B31" s="38"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="46"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="39"/>
-      <c r="I31" s="40"/>
-      <c r="J31" s="25"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="10"/>
+      <c r="A31" s="9"/>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="45"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="39"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="26"/>
+      <c r="L31" s="9"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="46"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="39"/>
-      <c r="I32" s="40"/>
-      <c r="J32" s="25"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="10"/>
-    </row>
-    <row r="33" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="11"/>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="46"/>
-      <c r="F33" s="46"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="24"/>
-      <c r="L33" s="10"/>
+      <c r="A32" s="9"/>
+      <c r="B32" s="37"/>
+      <c r="C32" s="37"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="45"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="39"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="9"/>
+    </row>
+    <row r="33" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="45"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="22"/>
+      <c r="K33" s="23"/>
+      <c r="L33" s="9"/>
     </row>
     <row r="34" spans="1:12" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10"/>
-      <c r="L34" s="10"/>
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
     </row>
     <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10"/>
-      <c r="B35" s="43" t="s">
+      <c r="A35" s="9"/>
+      <c r="B35" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="44"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="83"/>
-      <c r="F35" s="83"/>
-      <c r="G35" s="83"/>
-      <c r="H35" s="83"/>
-      <c r="I35" s="83"/>
-      <c r="J35" s="83"/>
-      <c r="K35" s="83"/>
-      <c r="L35" s="10"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="82"/>
+      <c r="F35" s="82"/>
+      <c r="G35" s="82"/>
+      <c r="H35" s="82"/>
+      <c r="I35" s="82"/>
+      <c r="J35" s="82"/>
+      <c r="K35" s="82"/>
+      <c r="L35" s="9"/>
     </row>
     <row r="36" spans="1:12" ht="1.1499999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="10"/>
+      <c r="A36" s="9"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
     </row>
     <row r="37" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="10"/>
-      <c r="B37" s="28"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="41"/>
-      <c r="E37" s="41"/>
-      <c r="F37" s="42"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="39"/>
-      <c r="I37" s="40"/>
-      <c r="J37" s="28"/>
-      <c r="K37" s="29"/>
-      <c r="L37" s="10"/>
+      <c r="A37" s="9"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="40"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="41"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="39"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="9"/>
     </row>
     <row r="38" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="10"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="41"/>
-      <c r="E38" s="41"/>
-      <c r="F38" s="42"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="39"/>
-      <c r="I38" s="40"/>
-      <c r="J38" s="28"/>
-      <c r="K38" s="29"/>
-      <c r="L38" s="10"/>
+      <c r="A38" s="9"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="40"/>
+      <c r="E38" s="40"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="39"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="9"/>
     </row>
     <row r="39" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10"/>
-      <c r="B39" s="47"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="42"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="39"/>
-      <c r="I39" s="40"/>
-      <c r="J39" s="28"/>
-      <c r="K39" s="29"/>
-      <c r="L39" s="10"/>
+      <c r="A39" s="9"/>
+      <c r="B39" s="46"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="39"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="28"/>
+      <c r="L39" s="9"/>
     </row>
     <row r="40" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10"/>
-      <c r="B40" s="47"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="42"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="39"/>
-      <c r="I40" s="40"/>
-      <c r="J40" s="28"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="10"/>
+      <c r="A40" s="9"/>
+      <c r="B40" s="46"/>
+      <c r="C40" s="46"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="41"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="39"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="28"/>
+      <c r="L40" s="9"/>
     </row>
     <row r="41" spans="1:12" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="10"/>
-      <c r="H41" s="10"/>
-      <c r="I41" s="10"/>
-      <c r="J41" s="10"/>
-      <c r="K41" s="10"/>
-      <c r="L41" s="10"/>
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+      <c r="I41" s="9"/>
+      <c r="J41" s="9"/>
+      <c r="K41" s="9"/>
+      <c r="L41" s="9"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A42" s="10"/>
-      <c r="B42" s="78" t="s">
+      <c r="A42" s="9"/>
+      <c r="B42" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="79"/>
-      <c r="D42" s="79"/>
-      <c r="E42" s="79"/>
-      <c r="F42" s="79"/>
-      <c r="G42" s="79"/>
-      <c r="H42" s="79"/>
-      <c r="I42" s="79"/>
-      <c r="J42" s="79"/>
-      <c r="K42" s="80"/>
-      <c r="L42" s="10"/>
+      <c r="C42" s="78"/>
+      <c r="D42" s="78"/>
+      <c r="E42" s="78"/>
+      <c r="F42" s="78"/>
+      <c r="G42" s="78"/>
+      <c r="H42" s="78"/>
+      <c r="I42" s="78"/>
+      <c r="J42" s="78"/>
+      <c r="K42" s="79"/>
+      <c r="L42" s="9"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A43" s="10"/>
-      <c r="B43" s="32"/>
-      <c r="C43" s="33"/>
-      <c r="D43" s="33"/>
-      <c r="E43" s="33"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="33"/>
-      <c r="H43" s="33"/>
-      <c r="I43" s="33"/>
-      <c r="J43" s="33"/>
-      <c r="K43" s="34"/>
-      <c r="L43" s="10"/>
+      <c r="A43" s="9"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="32"/>
+      <c r="J43" s="32"/>
+      <c r="K43" s="33"/>
+      <c r="L43" s="9"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A44" s="10"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="33"/>
-      <c r="D44" s="33"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="33"/>
-      <c r="G44" s="33"/>
-      <c r="H44" s="33"/>
-      <c r="I44" s="33"/>
-      <c r="J44" s="33"/>
-      <c r="K44" s="34"/>
-      <c r="L44" s="10"/>
+      <c r="A44" s="9"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
+      <c r="K44" s="33"/>
+      <c r="L44" s="9"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A45" s="10"/>
-      <c r="B45" s="32"/>
-      <c r="C45" s="33"/>
-      <c r="D45" s="33"/>
-      <c r="E45" s="33"/>
-      <c r="F45" s="33"/>
-      <c r="G45" s="33"/>
-      <c r="H45" s="33"/>
-      <c r="I45" s="33"/>
-      <c r="J45" s="33"/>
-      <c r="K45" s="34"/>
-      <c r="L45" s="10"/>
+      <c r="A45" s="9"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="32"/>
+      <c r="J45" s="32"/>
+      <c r="K45" s="33"/>
+      <c r="L45" s="9"/>
     </row>
     <row r="46" spans="1:12" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="10"/>
-      <c r="B46" s="35"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="36"/>
-      <c r="E46" s="36"/>
-      <c r="F46" s="36"/>
-      <c r="G46" s="36"/>
-      <c r="H46" s="36"/>
-      <c r="I46" s="36"/>
-      <c r="J46" s="36"/>
-      <c r="K46" s="37"/>
-      <c r="L46" s="10"/>
+      <c r="A46" s="9"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="35"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="35"/>
+      <c r="I46" s="35"/>
+      <c r="J46" s="35"/>
+      <c r="K46" s="36"/>
+      <c r="L46" s="9"/>
     </row>
     <row r="47" spans="1:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="10"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="12"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
-      <c r="L47" s="10"/>
+      <c r="A47" s="9"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="11"/>
+      <c r="G47" s="11"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+      <c r="J47" s="11"/>
+      <c r="K47" s="11"/>
+      <c r="L47" s="9"/>
     </row>
     <row r="48" spans="1:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="10"/>
-      <c r="B48" s="30" t="s">
+      <c r="A48" s="9"/>
+      <c r="B48" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="30"/>
-      <c r="F48" s="30"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="30"/>
-      <c r="I48" s="30"/>
-      <c r="J48" s="30"/>
-      <c r="K48" s="30"/>
-      <c r="L48" s="10"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="29"/>
+      <c r="J48" s="29"/>
+      <c r="K48" s="29"/>
+      <c r="L48" s="9"/>
     </row>
     <row r="49" spans="1:24" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="10"/>
-      <c r="B49" s="30" t="s">
+      <c r="A49" s="9"/>
+      <c r="B49" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="30"/>
-      <c r="F49" s="30"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="30"/>
-      <c r="I49" s="30"/>
-      <c r="J49" s="30"/>
-      <c r="K49" s="30"/>
-      <c r="L49" s="10"/>
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="29"/>
+      <c r="F49" s="29"/>
+      <c r="G49" s="29"/>
+      <c r="H49" s="29"/>
+      <c r="I49" s="29"/>
+      <c r="J49" s="29"/>
+      <c r="K49" s="29"/>
+      <c r="L49" s="9"/>
     </row>
     <row r="50" spans="1:24" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="10"/>
-      <c r="B50" s="14" t="s">
+      <c r="A50" s="9"/>
+      <c r="B50" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="14"/>
-      <c r="J50" s="14"/>
-      <c r="K50" s="14"/>
-      <c r="L50" s="10"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="13"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="13"/>
+      <c r="K50" s="13"/>
+      <c r="L50" s="9"/>
     </row>
     <row r="51" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A51" s="10"/>
-      <c r="B51" s="31" t="s">
+      <c r="A51" s="9"/>
+      <c r="B51" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="C51" s="31"/>
-      <c r="D51" s="31"/>
-      <c r="E51" s="31"/>
-      <c r="F51" s="31"/>
-      <c r="G51" s="31"/>
-      <c r="H51" s="31"/>
-      <c r="I51" s="31"/>
-      <c r="J51" s="31"/>
-      <c r="K51" s="31"/>
-      <c r="L51" s="10"/>
+      <c r="C51" s="30"/>
+      <c r="D51" s="30"/>
+      <c r="E51" s="30"/>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+      <c r="H51" s="30"/>
+      <c r="I51" s="30"/>
+      <c r="J51" s="30"/>
+      <c r="K51" s="30"/>
+      <c r="L51" s="9"/>
     </row>
     <row r="52" spans="1:24" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="10"/>
-      <c r="B52" s="31"/>
-      <c r="C52" s="31"/>
-      <c r="D52" s="31"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="31"/>
-      <c r="G52" s="31"/>
-      <c r="H52" s="31"/>
-      <c r="I52" s="31"/>
-      <c r="J52" s="31"/>
-      <c r="K52" s="31"/>
-      <c r="L52" s="10"/>
+      <c r="A52" s="9"/>
+      <c r="B52" s="30"/>
+      <c r="C52" s="30"/>
+      <c r="D52" s="30"/>
+      <c r="E52" s="30"/>
+      <c r="F52" s="30"/>
+      <c r="G52" s="30"/>
+      <c r="H52" s="30"/>
+      <c r="I52" s="30"/>
+      <c r="J52" s="30"/>
+      <c r="K52" s="30"/>
+      <c r="L52" s="9"/>
     </row>
     <row r="53" spans="1:24" ht="15" x14ac:dyDescent="0.25">
-      <c r="T53" s="21"/>
-      <c r="U53" s="21"/>
-      <c r="V53" s="21"/>
-      <c r="W53" s="21"/>
-      <c r="X53" s="21"/>
+      <c r="T53" s="20"/>
+      <c r="U53" s="20"/>
+      <c r="V53" s="20"/>
+      <c r="W53" s="20"/>
+      <c r="X53" s="20"/>
     </row>
     <row r="54" spans="1:24" ht="15" x14ac:dyDescent="0.25">
-      <c r="T54" s="21"/>
-      <c r="U54" s="21"/>
-      <c r="V54" s="21"/>
-      <c r="W54" s="21"/>
-      <c r="X54" s="21"/>
+      <c r="T54" s="20"/>
+      <c r="U54" s="20"/>
+      <c r="V54" s="20"/>
+      <c r="W54" s="20"/>
+      <c r="X54" s="20"/>
     </row>
     <row r="55" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="T55" s="22"/>
-      <c r="U55" s="22"/>
-      <c r="V55" s="22"/>
-      <c r="W55" s="22"/>
-      <c r="X55" s="22"/>
+      <c r="T55" s="21"/>
+      <c r="U55" s="21"/>
+      <c r="V55" s="21"/>
+      <c r="W55" s="21"/>
+      <c r="X55" s="21"/>
     </row>
     <row r="56" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="22"/>
-      <c r="T56" s="22"/>
-      <c r="U56" s="22"/>
-      <c r="V56" s="22"/>
-      <c r="W56" s="22"/>
-      <c r="X56" s="22"/>
+      <c r="E56" s="21"/>
+      <c r="F56" s="21"/>
+      <c r="G56" s="21"/>
+      <c r="H56" s="21"/>
+      <c r="T56" s="21"/>
+      <c r="U56" s="21"/>
+      <c r="V56" s="21"/>
+      <c r="W56" s="21"/>
+      <c r="X56" s="21"/>
     </row>
     <row r="57" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="E57" s="22"/>
-      <c r="F57" s="22"/>
-      <c r="G57" s="22"/>
-      <c r="H57" s="22"/>
-      <c r="T57" s="22"/>
-      <c r="U57" s="22"/>
-      <c r="V57" s="22"/>
-      <c r="W57" s="22"/>
-      <c r="X57" s="22"/>
+      <c r="E57" s="21"/>
+      <c r="F57" s="21"/>
+      <c r="G57" s="21"/>
+      <c r="H57" s="21"/>
+      <c r="T57" s="21"/>
+      <c r="U57" s="21"/>
+      <c r="V57" s="21"/>
+      <c r="W57" s="21"/>
+      <c r="X57" s="21"/>
     </row>
     <row r="58" spans="1:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D58" s="9"/>
-      <c r="E58" s="77"/>
-      <c r="F58" s="77"/>
-      <c r="G58" s="77"/>
-      <c r="H58" s="77"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="76"/>
+      <c r="F58" s="76"/>
+      <c r="G58" s="76"/>
+      <c r="H58" s="76"/>
     </row>
     <row r="59" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B59" s="76"/>
-      <c r="C59" s="76"/>
-      <c r="D59" s="76"/>
-      <c r="E59" s="76"/>
-      <c r="G59" s="76"/>
-      <c r="H59" s="76"/>
-      <c r="I59" s="76"/>
-      <c r="J59" s="76"/>
+      <c r="B59" s="75"/>
+      <c r="C59" s="75"/>
+      <c r="D59" s="75"/>
+      <c r="E59" s="75"/>
+      <c r="G59" s="75"/>
+      <c r="H59" s="75"/>
+      <c r="I59" s="75"/>
+      <c r="J59" s="75"/>
     </row>
     <row r="60" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B60" s="22" t="s">
+      <c r="B60" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C60" s="21"/>
+      <c r="D60" s="21"/>
+      <c r="E60" s="21"/>
+      <c r="G60" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="H60" s="21"/>
+      <c r="I60" s="21"/>
+      <c r="J60" s="21"/>
+    </row>
+    <row r="61" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B61" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="G60" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="H60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
-    </row>
-    <row r="61" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B61" s="22" t="s">
+      <c r="C61" s="21"/>
+      <c r="D61" s="21"/>
+      <c r="E61" s="21"/>
+      <c r="G61" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C61" s="22"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="G61" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="H61" s="22"/>
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
+      <c r="H61" s="21"/>
+      <c r="I61" s="21"/>
+      <c r="J61" s="21"/>
     </row>
     <row r="64" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="67" t="s">
+      <c r="A64" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="B64" s="67"/>
-      <c r="C64" s="67"/>
-      <c r="D64" s="67" t="s">
+      <c r="B64" s="66"/>
+      <c r="C64" s="66"/>
+      <c r="D64" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="E64" s="67"/>
-      <c r="F64" s="67"/>
-      <c r="G64" s="67"/>
-      <c r="H64" s="67"/>
-      <c r="I64" s="9"/>
-      <c r="J64" s="8" t="s">
+      <c r="E64" s="66"/>
+      <c r="F64" s="66"/>
+      <c r="G64" s="66"/>
+      <c r="H64" s="66"/>
+      <c r="I64" s="8"/>
+      <c r="J64" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="K64" s="9"/>
+      <c r="K64" s="8"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A65" s="9"/>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="67" t="s">
+      <c r="A65" s="8"/>
+      <c r="B65" s="8"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="E65" s="67"/>
-      <c r="F65" s="67"/>
-      <c r="G65" s="67"/>
-      <c r="H65" s="67"/>
-      <c r="I65" s="9"/>
-      <c r="J65" s="18" t="s">
+      <c r="E65" s="66"/>
+      <c r="F65" s="66"/>
+      <c r="G65" s="66"/>
+      <c r="H65" s="66"/>
+      <c r="I65" s="8"/>
+      <c r="J65" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="K65" s="9"/>
+      <c r="K65" s="8"/>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A66" s="9"/>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="9"/>
-      <c r="H66" s="9"/>
-      <c r="I66" s="9"/>
-      <c r="J66" s="9"/>
-      <c r="K66" s="9"/>
+      <c r="A66" s="8"/>
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="8"/>
+      <c r="G66" s="8"/>
+      <c r="H66" s="8"/>
+      <c r="I66" s="8"/>
+      <c r="J66" s="8"/>
+      <c r="K66" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="94">

</xml_diff>

<commit_message>
Version 1.3 del sistema de laboratorio
</commit_message>
<xml_diff>
--- a/modules/laboratorio/muestra/plantilla/CSJ-DRDYCS-LAYS – R - 1-RESULTADOS ANALISIS DE  SUELOS.xlsx
+++ b/modules/laboratorio/muestra/plantilla/CSJ-DRDYCS-LAYS – R - 1-RESULTADOS ANALISIS DE  SUELOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SISTEMAS\gestionTI2026\modules\laboratorio\muestra\plantilla\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678C2917-050B-4645-B4D5-5DAE53521E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D980814D-724D-4B04-8104-A75E02CFD4FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="9915" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO 001 -2024 " sheetId="2" r:id="rId1"/>
@@ -350,7 +350,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -363,8 +363,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="37">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -808,11 +814,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -859,9 +889,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="17" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -871,6 +898,27 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -898,6 +946,15 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -931,50 +988,62 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="33" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1057,8 +1126,11 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1484,8 +1556,8 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1493,14 +1565,14 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="65" t="s">
+      <c r="J2" s="78" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="66"/>
+      <c r="K2" s="79"/>
     </row>
     <row r="3" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
       <c r="D3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1508,12 +1580,12 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="65"/>
-      <c r="K3" s="67"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="80"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
       <c r="D4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1523,8 +1595,8 @@
       <c r="I4" s="7"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
       <c r="D5" s="5" t="s">
         <v>3</v>
       </c>
@@ -1535,33 +1607,33 @@
     </row>
     <row r="6" spans="1:12" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:12" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="B7" s="68" t="s">
+      <c r="B7" s="81" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
-      <c r="F7" s="68"/>
-      <c r="G7" s="68"/>
-      <c r="H7" s="68"/>
-      <c r="I7" s="68"/>
-      <c r="J7" s="68"/>
-      <c r="K7" s="68"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="81"/>
+      <c r="E7" s="81"/>
+      <c r="F7" s="81"/>
+      <c r="G7" s="81"/>
+      <c r="H7" s="81"/>
+      <c r="I7" s="81"/>
+      <c r="J7" s="81"/>
+      <c r="K7" s="81"/>
     </row>
     <row r="8" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
-      <c r="B8" s="61" t="s">
+      <c r="B8" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="74"/>
+      <c r="K8" s="74"/>
       <c r="L8" s="9"/>
     </row>
     <row r="9" spans="1:12" ht="7.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1580,10 +1652,10 @@
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9"/>
-      <c r="B10" s="55" t="s">
+      <c r="B10" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="56"/>
+      <c r="C10" s="69"/>
       <c r="D10" s="1" t="s">
         <v>5</v>
       </c>
@@ -1609,8 +1681,8 @@
       <c r="D11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
@@ -1618,20 +1690,20 @@
       <c r="K11" s="9"/>
       <c r="L11" s="9"/>
     </row>
-    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9"/>
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="57"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="59"/>
-      <c r="F12" s="59"/>
-      <c r="G12" s="59"/>
-      <c r="H12" s="59"/>
-      <c r="I12" s="59"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="60"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="71"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="72"/>
+      <c r="K12" s="73"/>
       <c r="L12" s="9"/>
     </row>
     <row r="13" spans="1:12" ht="4.1500000000000004" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1648,21 +1720,21 @@
       <c r="K13" s="9"/>
       <c r="L13" s="9"/>
     </row>
-    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9"/>
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="57"/>
-      <c r="D14" s="61" t="s">
+      <c r="C14" s="70"/>
+      <c r="D14" s="74" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="61"/>
+      <c r="E14" s="74"/>
       <c r="F14" s="2"/>
-      <c r="G14" s="61" t="s">
+      <c r="G14" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="61"/>
+      <c r="H14" s="74"/>
       <c r="I14" s="2"/>
       <c r="J14" s="1" t="s">
         <v>29</v>
@@ -1684,20 +1756,20 @@
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
     </row>
-    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9"/>
-      <c r="B16" s="55" t="s">
+      <c r="B16" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="59"/>
-      <c r="H16" s="59"/>
-      <c r="I16" s="59"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="60"/>
+      <c r="C16" s="70"/>
+      <c r="D16" s="71"/>
+      <c r="E16" s="72"/>
+      <c r="F16" s="72"/>
+      <c r="G16" s="72"/>
+      <c r="H16" s="72"/>
+      <c r="I16" s="72"/>
+      <c r="J16" s="72"/>
+      <c r="K16" s="73"/>
       <c r="L16" s="9"/>
     </row>
     <row r="17" spans="1:12" ht="3" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1716,23 +1788,23 @@
     </row>
     <row r="18" spans="1:12" ht="13.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9"/>
-      <c r="B18" s="55" t="s">
+      <c r="B18" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="56"/>
-      <c r="D18" s="18" t="s">
+      <c r="C18" s="69"/>
+      <c r="D18" s="17" t="s">
         <v>32</v>
       </c>
       <c r="E18" s="2"/>
-      <c r="F18" s="63" t="s">
+      <c r="F18" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="G18" s="64"/>
+      <c r="G18" s="77"/>
       <c r="H18" s="2"/>
-      <c r="I18" s="63" t="s">
+      <c r="I18" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="J18" s="64"/>
+      <c r="J18" s="77"/>
       <c r="K18" s="2"/>
       <c r="L18" s="9"/>
     </row>
@@ -1752,20 +1824,20 @@
     </row>
     <row r="20" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="57"/>
-      <c r="D20" s="58"/>
-      <c r="E20" s="59"/>
-      <c r="F20" s="62" t="s">
+      <c r="C20" s="70"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="72"/>
+      <c r="F20" s="75" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="62"/>
-      <c r="H20" s="62"/>
-      <c r="I20" s="62"/>
-      <c r="J20" s="59"/>
-      <c r="K20" s="59"/>
+      <c r="G20" s="75"/>
+      <c r="H20" s="75"/>
+      <c r="I20" s="75"/>
+      <c r="J20" s="72"/>
+      <c r="K20" s="72"/>
       <c r="L20" s="9"/>
     </row>
     <row r="21" spans="1:12" ht="4.1500000000000004" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1784,25 +1856,25 @@
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
-      <c r="B22" s="55" t="s">
+      <c r="B22" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="56"/>
+      <c r="C22" s="69"/>
       <c r="D22" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="58"/>
-      <c r="F22" s="59"/>
-      <c r="G22" s="60"/>
+      <c r="E22" s="71"/>
+      <c r="F22" s="72"/>
+      <c r="G22" s="73"/>
       <c r="H22" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="I22" s="59"/>
-      <c r="J22" s="59"/>
-      <c r="K22" s="59"/>
+      <c r="I22" s="72"/>
+      <c r="J22" s="72"/>
+      <c r="K22" s="72"/>
       <c r="L22" s="9"/>
     </row>
-    <row r="23" spans="1:12" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -1816,42 +1888,42 @@
       <c r="K23" s="9"/>
       <c r="L23" s="9"/>
     </row>
-    <row r="24" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
-      <c r="B24" s="69" t="s">
+      <c r="B24" s="82" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="70"/>
-      <c r="D24" s="80" t="s">
+      <c r="C24" s="83"/>
+      <c r="D24" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="80"/>
-      <c r="F24" s="80"/>
-      <c r="G24" s="47" t="s">
+      <c r="E24" s="93"/>
+      <c r="F24" s="93"/>
+      <c r="G24" s="95" t="s">
         <v>18</v>
       </c>
-      <c r="H24" s="49" t="s">
+      <c r="H24" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="50"/>
-      <c r="J24" s="49" t="s">
+      <c r="I24" s="61"/>
+      <c r="J24" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="K24" s="73"/>
+      <c r="K24" s="86"/>
       <c r="L24" s="9"/>
     </row>
-    <row r="25" spans="1:12" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9"/>
-      <c r="B25" s="71"/>
-      <c r="C25" s="72"/>
-      <c r="D25" s="81"/>
-      <c r="E25" s="81"/>
-      <c r="F25" s="81"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="52"/>
-      <c r="J25" s="51"/>
-      <c r="K25" s="74"/>
+      <c r="B25" s="84"/>
+      <c r="C25" s="85"/>
+      <c r="D25" s="94"/>
+      <c r="E25" s="94"/>
+      <c r="F25" s="94"/>
+      <c r="G25" s="96"/>
+      <c r="H25" s="62"/>
+      <c r="I25" s="63"/>
+      <c r="J25" s="62"/>
+      <c r="K25" s="87"/>
       <c r="L25" s="9"/>
     </row>
     <row r="26" spans="1:12" ht="2.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1868,23 +1940,23 @@
       <c r="K26" s="9"/>
       <c r="L26" s="9"/>
     </row>
-    <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9"/>
-      <c r="B27" s="42" t="s">
+      <c r="B27" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="43"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="82"/>
-      <c r="F27" s="82"/>
-      <c r="G27" s="82"/>
-      <c r="H27" s="82"/>
-      <c r="I27" s="82"/>
-      <c r="J27" s="82"/>
-      <c r="K27" s="82"/>
+      <c r="C27" s="67"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="67"/>
+      <c r="F27" s="67"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="67"/>
+      <c r="J27" s="67"/>
+      <c r="K27" s="67"/>
       <c r="L27" s="9"/>
     </row>
-    <row r="28" spans="1:12" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -1900,78 +1972,78 @@
     </row>
     <row r="29" spans="1:12" s="4" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
       <c r="G29" s="12"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="26"/>
+      <c r="H29" s="64"/>
+      <c r="I29" s="65"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="32"/>
       <c r="L29" s="9"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
-      <c r="B30" s="37"/>
-      <c r="C30" s="37"/>
-      <c r="D30" s="44"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="45"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
       <c r="G30" s="12"/>
-      <c r="H30" s="38"/>
-      <c r="I30" s="39"/>
-      <c r="J30" s="24"/>
-      <c r="K30" s="26"/>
+      <c r="H30" s="47"/>
+      <c r="I30" s="48"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="32"/>
       <c r="L30" s="9"/>
     </row>
     <row r="31" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
-      <c r="B31" s="37"/>
-      <c r="C31" s="37"/>
-      <c r="D31" s="44"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
       <c r="G31" s="12"/>
-      <c r="H31" s="38"/>
-      <c r="I31" s="39"/>
-      <c r="J31" s="24"/>
-      <c r="K31" s="26"/>
+      <c r="H31" s="47"/>
+      <c r="I31" s="48"/>
+      <c r="J31" s="30"/>
+      <c r="K31" s="32"/>
       <c r="L31" s="9"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
-      <c r="B32" s="37"/>
-      <c r="C32" s="37"/>
-      <c r="D32" s="44"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="45"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="55"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="56"/>
       <c r="G32" s="12"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="39"/>
-      <c r="J32" s="24"/>
-      <c r="K32" s="25"/>
+      <c r="H32" s="47"/>
+      <c r="I32" s="48"/>
+      <c r="J32" s="30"/>
+      <c r="K32" s="31"/>
       <c r="L32" s="9"/>
     </row>
     <row r="33" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
-      <c r="B33" s="37"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="45"/>
+      <c r="B33" s="46"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="56"/>
       <c r="G33" s="12"/>
-      <c r="H33" s="38"/>
-      <c r="I33" s="39"/>
-      <c r="J33" s="22"/>
-      <c r="K33" s="23"/>
+      <c r="H33" s="47"/>
+      <c r="I33" s="48"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="29"/>
       <c r="L33" s="9"/>
     </row>
     <row r="34" spans="1:12" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9"/>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
+      <c r="B34" s="57"/>
+      <c r="C34" s="57"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
@@ -1982,90 +2054,90 @@
       <c r="K34" s="9"/>
       <c r="L34" s="9"/>
     </row>
-    <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9"/>
-      <c r="B35" s="42" t="s">
+    <row r="35" spans="1:12" s="24" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="23"/>
+      <c r="B35" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="43"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="82"/>
-      <c r="F35" s="82"/>
-      <c r="G35" s="82"/>
-      <c r="H35" s="82"/>
-      <c r="I35" s="82"/>
-      <c r="J35" s="82"/>
-      <c r="K35" s="82"/>
-      <c r="L35" s="9"/>
-    </row>
-    <row r="36" spans="1:12" ht="1.1499999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="9"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="9"/>
-      <c r="L36" s="9"/>
+      <c r="C35" s="59"/>
+      <c r="D35" s="59"/>
+      <c r="E35" s="59"/>
+      <c r="F35" s="59"/>
+      <c r="G35" s="59"/>
+      <c r="H35" s="59"/>
+      <c r="I35" s="59"/>
+      <c r="J35" s="59"/>
+      <c r="K35" s="59"/>
+      <c r="L35" s="23"/>
+    </row>
+    <row r="36" spans="1:12" s="24" customFormat="1" ht="3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="23"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="23"/>
     </row>
     <row r="37" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
-      <c r="B37" s="27"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="40"/>
-      <c r="E37" s="40"/>
-      <c r="F37" s="41"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="39"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="28"/>
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="53"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="53"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="51"/>
+      <c r="J37" s="37"/>
+      <c r="K37" s="37"/>
       <c r="L37" s="9"/>
     </row>
     <row r="38" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
-      <c r="B38" s="27"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="40"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="38"/>
-      <c r="I38" s="39"/>
-      <c r="J38" s="27"/>
-      <c r="K38" s="28"/>
+      <c r="B38" s="35"/>
+      <c r="C38" s="36"/>
+      <c r="D38" s="52"/>
+      <c r="E38" s="52"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="22"/>
+      <c r="H38" s="49"/>
+      <c r="I38" s="50"/>
+      <c r="J38" s="35"/>
+      <c r="K38" s="36"/>
       <c r="L38" s="9"/>
     </row>
     <row r="39" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
-      <c r="B39" s="46"/>
-      <c r="C39" s="46"/>
-      <c r="D39" s="40"/>
-      <c r="E39" s="40"/>
-      <c r="F39" s="41"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="54"/>
       <c r="G39" s="12"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="39"/>
-      <c r="J39" s="27"/>
-      <c r="K39" s="28"/>
+      <c r="H39" s="47"/>
+      <c r="I39" s="48"/>
+      <c r="J39" s="33"/>
+      <c r="K39" s="34"/>
       <c r="L39" s="9"/>
     </row>
     <row r="40" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
-      <c r="B40" s="46"/>
-      <c r="C40" s="46"/>
-      <c r="D40" s="40"/>
-      <c r="E40" s="40"/>
-      <c r="F40" s="41"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="53"/>
+      <c r="E40" s="53"/>
+      <c r="F40" s="54"/>
       <c r="G40" s="12"/>
-      <c r="H40" s="38"/>
-      <c r="I40" s="39"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="28"/>
+      <c r="H40" s="47"/>
+      <c r="I40" s="48"/>
+      <c r="J40" s="33"/>
+      <c r="K40" s="34"/>
       <c r="L40" s="9"/>
     </row>
     <row r="41" spans="1:12" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2084,74 +2156,74 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
-      <c r="B42" s="77" t="s">
+      <c r="B42" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="78"/>
-      <c r="D42" s="78"/>
-      <c r="E42" s="78"/>
-      <c r="F42" s="78"/>
-      <c r="G42" s="78"/>
-      <c r="H42" s="78"/>
-      <c r="I42" s="78"/>
-      <c r="J42" s="78"/>
-      <c r="K42" s="79"/>
+      <c r="C42" s="91"/>
+      <c r="D42" s="91"/>
+      <c r="E42" s="91"/>
+      <c r="F42" s="91"/>
+      <c r="G42" s="91"/>
+      <c r="H42" s="91"/>
+      <c r="I42" s="91"/>
+      <c r="J42" s="91"/>
+      <c r="K42" s="92"/>
       <c r="L42" s="9"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
-      <c r="B43" s="31"/>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="32"/>
-      <c r="J43" s="32"/>
-      <c r="K43" s="33"/>
+      <c r="B43" s="40"/>
+      <c r="C43" s="41"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="41"/>
+      <c r="H43" s="41"/>
+      <c r="I43" s="41"/>
+      <c r="J43" s="41"/>
+      <c r="K43" s="42"/>
       <c r="L43" s="9"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
-      <c r="B44" s="31"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="32"/>
-      <c r="J44" s="32"/>
-      <c r="K44" s="33"/>
+      <c r="B44" s="40"/>
+      <c r="C44" s="41"/>
+      <c r="D44" s="41"/>
+      <c r="E44" s="41"/>
+      <c r="F44" s="41"/>
+      <c r="G44" s="41"/>
+      <c r="H44" s="41"/>
+      <c r="I44" s="41"/>
+      <c r="J44" s="41"/>
+      <c r="K44" s="42"/>
       <c r="L44" s="9"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
-      <c r="B45" s="31"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="32"/>
-      <c r="J45" s="32"/>
-      <c r="K45" s="33"/>
+      <c r="B45" s="40"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="41"/>
+      <c r="F45" s="41"/>
+      <c r="G45" s="41"/>
+      <c r="H45" s="41"/>
+      <c r="I45" s="41"/>
+      <c r="J45" s="41"/>
+      <c r="K45" s="42"/>
       <c r="L45" s="9"/>
     </row>
-    <row r="46" spans="1:12" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="35"/>
-      <c r="J46" s="35"/>
-      <c r="K46" s="36"/>
+      <c r="B46" s="43"/>
+      <c r="C46" s="44"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="44"/>
+      <c r="F46" s="44"/>
+      <c r="G46" s="44"/>
+      <c r="H46" s="44"/>
+      <c r="I46" s="44"/>
+      <c r="J46" s="44"/>
+      <c r="K46" s="45"/>
       <c r="L46" s="9"/>
     </row>
     <row r="47" spans="1:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2170,34 +2242,34 @@
     </row>
     <row r="48" spans="1:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
-      <c r="B48" s="29" t="s">
+      <c r="B48" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C48" s="29"/>
-      <c r="D48" s="29"/>
-      <c r="E48" s="29"/>
-      <c r="F48" s="29"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="29"/>
-      <c r="I48" s="29"/>
-      <c r="J48" s="29"/>
-      <c r="K48" s="29"/>
+      <c r="C48" s="38"/>
+      <c r="D48" s="38"/>
+      <c r="E48" s="38"/>
+      <c r="F48" s="38"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="38"/>
+      <c r="J48" s="38"/>
+      <c r="K48" s="38"/>
       <c r="L48" s="9"/>
     </row>
     <row r="49" spans="1:24" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="C49" s="29"/>
-      <c r="D49" s="29"/>
-      <c r="E49" s="29"/>
-      <c r="F49" s="29"/>
-      <c r="G49" s="29"/>
-      <c r="H49" s="29"/>
-      <c r="I49" s="29"/>
-      <c r="J49" s="29"/>
-      <c r="K49" s="29"/>
+      <c r="C49" s="38"/>
+      <c r="D49" s="38"/>
+      <c r="E49" s="38"/>
+      <c r="F49" s="38"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="38"/>
+      <c r="I49" s="38"/>
+      <c r="J49" s="38"/>
+      <c r="K49" s="38"/>
       <c r="L49" s="9"/>
     </row>
     <row r="50" spans="1:24" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2218,135 +2290,135 @@
     </row>
     <row r="51" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A51" s="9"/>
-      <c r="B51" s="30" t="s">
+      <c r="B51" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="C51" s="30"/>
-      <c r="D51" s="30"/>
-      <c r="E51" s="30"/>
-      <c r="F51" s="30"/>
-      <c r="G51" s="30"/>
-      <c r="H51" s="30"/>
-      <c r="I51" s="30"/>
-      <c r="J51" s="30"/>
-      <c r="K51" s="30"/>
+      <c r="C51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="39"/>
+      <c r="G51" s="39"/>
+      <c r="H51" s="39"/>
+      <c r="I51" s="39"/>
+      <c r="J51" s="39"/>
+      <c r="K51" s="39"/>
       <c r="L51" s="9"/>
     </row>
     <row r="52" spans="1:24" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="30"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="30"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="30"/>
-      <c r="I52" s="30"/>
-      <c r="J52" s="30"/>
-      <c r="K52" s="30"/>
+      <c r="B52" s="39"/>
+      <c r="C52" s="39"/>
+      <c r="D52" s="39"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="39"/>
+      <c r="I52" s="39"/>
+      <c r="J52" s="39"/>
+      <c r="K52" s="39"/>
       <c r="L52" s="9"/>
     </row>
     <row r="53" spans="1:24" ht="15" x14ac:dyDescent="0.25">
-      <c r="T53" s="20"/>
-      <c r="U53" s="20"/>
-      <c r="V53" s="20"/>
-      <c r="W53" s="20"/>
-      <c r="X53" s="20"/>
+      <c r="T53" s="26"/>
+      <c r="U53" s="26"/>
+      <c r="V53" s="26"/>
+      <c r="W53" s="26"/>
+      <c r="X53" s="26"/>
     </row>
     <row r="54" spans="1:24" ht="15" x14ac:dyDescent="0.25">
-      <c r="T54" s="20"/>
-      <c r="U54" s="20"/>
-      <c r="V54" s="20"/>
-      <c r="W54" s="20"/>
-      <c r="X54" s="20"/>
+      <c r="T54" s="26"/>
+      <c r="U54" s="26"/>
+      <c r="V54" s="26"/>
+      <c r="W54" s="26"/>
+      <c r="X54" s="26"/>
     </row>
     <row r="55" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="T55" s="21"/>
-      <c r="U55" s="21"/>
-      <c r="V55" s="21"/>
-      <c r="W55" s="21"/>
-      <c r="X55" s="21"/>
+      <c r="T55" s="27"/>
+      <c r="U55" s="27"/>
+      <c r="V55" s="27"/>
+      <c r="W55" s="27"/>
+      <c r="X55" s="27"/>
     </row>
     <row r="56" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="E56" s="21"/>
-      <c r="F56" s="21"/>
-      <c r="G56" s="21"/>
-      <c r="H56" s="21"/>
-      <c r="T56" s="21"/>
-      <c r="U56" s="21"/>
-      <c r="V56" s="21"/>
-      <c r="W56" s="21"/>
-      <c r="X56" s="21"/>
+      <c r="E56" s="27"/>
+      <c r="F56" s="27"/>
+      <c r="G56" s="27"/>
+      <c r="H56" s="27"/>
+      <c r="T56" s="27"/>
+      <c r="U56" s="27"/>
+      <c r="V56" s="27"/>
+      <c r="W56" s="27"/>
+      <c r="X56" s="27"/>
     </row>
     <row r="57" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="E57" s="21"/>
-      <c r="F57" s="21"/>
-      <c r="G57" s="21"/>
-      <c r="H57" s="21"/>
-      <c r="T57" s="21"/>
-      <c r="U57" s="21"/>
-      <c r="V57" s="21"/>
-      <c r="W57" s="21"/>
-      <c r="X57" s="21"/>
+      <c r="E57" s="27"/>
+      <c r="F57" s="27"/>
+      <c r="G57" s="27"/>
+      <c r="H57" s="27"/>
+      <c r="T57" s="27"/>
+      <c r="U57" s="27"/>
+      <c r="V57" s="27"/>
+      <c r="W57" s="27"/>
+      <c r="X57" s="27"/>
     </row>
     <row r="58" spans="1:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D58" s="8"/>
-      <c r="E58" s="76"/>
-      <c r="F58" s="76"/>
-      <c r="G58" s="76"/>
-      <c r="H58" s="76"/>
+      <c r="E58" s="89"/>
+      <c r="F58" s="89"/>
+      <c r="G58" s="89"/>
+      <c r="H58" s="89"/>
     </row>
     <row r="59" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B59" s="75"/>
-      <c r="C59" s="75"/>
-      <c r="D59" s="75"/>
-      <c r="E59" s="75"/>
-      <c r="G59" s="75"/>
-      <c r="H59" s="75"/>
-      <c r="I59" s="75"/>
-      <c r="J59" s="75"/>
+      <c r="B59" s="88"/>
+      <c r="C59" s="88"/>
+      <c r="D59" s="88"/>
+      <c r="E59" s="88"/>
+      <c r="G59" s="88"/>
+      <c r="H59" s="88"/>
+      <c r="I59" s="88"/>
+      <c r="J59" s="88"/>
     </row>
     <row r="60" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B60" s="21" t="s">
+      <c r="B60" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="C60" s="21"/>
-      <c r="D60" s="21"/>
-      <c r="E60" s="21"/>
-      <c r="G60" s="21" t="s">
+      <c r="C60" s="27"/>
+      <c r="D60" s="27"/>
+      <c r="E60" s="27"/>
+      <c r="G60" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="H60" s="21"/>
-      <c r="I60" s="21"/>
-      <c r="J60" s="21"/>
+      <c r="H60" s="27"/>
+      <c r="I60" s="27"/>
+      <c r="J60" s="27"/>
     </row>
     <row r="61" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B61" s="21" t="s">
+      <c r="B61" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="C61" s="21"/>
-      <c r="D61" s="21"/>
-      <c r="E61" s="21"/>
-      <c r="G61" s="21" t="s">
+      <c r="C61" s="27"/>
+      <c r="D61" s="27"/>
+      <c r="E61" s="27"/>
+      <c r="G61" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="H61" s="21"/>
-      <c r="I61" s="21"/>
-      <c r="J61" s="21"/>
+      <c r="H61" s="27"/>
+      <c r="I61" s="27"/>
+      <c r="J61" s="27"/>
     </row>
     <row r="64" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="66" t="s">
+      <c r="A64" s="79" t="s">
         <v>43</v>
       </c>
-      <c r="B64" s="66"/>
-      <c r="C64" s="66"/>
-      <c r="D64" s="66" t="s">
+      <c r="B64" s="79"/>
+      <c r="C64" s="79"/>
+      <c r="D64" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="E64" s="66"/>
-      <c r="F64" s="66"/>
-      <c r="G64" s="66"/>
-      <c r="H64" s="66"/>
+      <c r="E64" s="79"/>
+      <c r="F64" s="79"/>
+      <c r="G64" s="79"/>
+      <c r="H64" s="79"/>
       <c r="I64" s="8"/>
       <c r="J64" s="7" t="s">
         <v>40</v>
@@ -2357,15 +2429,15 @@
       <c r="A65" s="8"/>
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
-      <c r="D65" s="66" t="s">
+      <c r="D65" s="79" t="s">
         <v>42</v>
       </c>
-      <c r="E65" s="66"/>
-      <c r="F65" s="66"/>
-      <c r="G65" s="66"/>
-      <c r="H65" s="66"/>
+      <c r="E65" s="79"/>
+      <c r="F65" s="79"/>
+      <c r="G65" s="79"/>
+      <c r="H65" s="79"/>
       <c r="I65" s="8"/>
-      <c r="J65" s="17" t="s">
+      <c r="J65" s="16" t="s">
         <v>41</v>
       </c>
       <c r="K65" s="8"/>
@@ -2384,7 +2456,7 @@
       <c r="K66" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="94">
+  <mergeCells count="93">
     <mergeCell ref="D64:H64"/>
     <mergeCell ref="E56:H56"/>
     <mergeCell ref="B42:K42"/>
@@ -2393,14 +2465,12 @@
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="D31:F31"/>
     <mergeCell ref="D32:F32"/>
-    <mergeCell ref="E27:K27"/>
     <mergeCell ref="J29:K29"/>
     <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="E35:K35"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="D37:F37"/>
+    <mergeCell ref="G24:G25"/>
     <mergeCell ref="I22:K22"/>
     <mergeCell ref="B24:C25"/>
     <mergeCell ref="J24:K25"/>
@@ -2437,24 +2507,25 @@
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G24:G25"/>
     <mergeCell ref="H24:I25"/>
     <mergeCell ref="H33:I33"/>
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="H29:I29"/>
+    <mergeCell ref="B27:K27"/>
     <mergeCell ref="H38:I38"/>
     <mergeCell ref="H37:I37"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="D39:F39"/>
-    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="D33:F33"/>
     <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:K35"/>
     <mergeCell ref="J33:K33"/>
     <mergeCell ref="J32:K32"/>
     <mergeCell ref="J31:K31"/>

</xml_diff>